<commit_message>
Lipeza de dados: retirada as células (valores) vazios
</commit_message>
<xml_diff>
--- a/datacleaning.xlsx
+++ b/datacleaning.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="34">
   <si>
     <t>duration</t>
   </si>
@@ -115,6 +115,9 @@
   </si>
   <si>
     <t>374.0</t>
+  </si>
+  <si>
+    <t>26122020</t>
   </si>
 </sst>
 </file>
@@ -150,9 +153,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -457,7 +461,7 @@
   <dimension ref="A1:E33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -918,8 +922,8 @@
       <c r="A28">
         <v>60</v>
       </c>
-      <c r="B28" s="1">
-        <v>44191</v>
+      <c r="B28" s="2" t="s">
+        <v>33</v>
       </c>
       <c r="C28">
         <v>100</v>
@@ -1015,6 +1019,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>